<commit_message>
added Control Flow Graph and Cyclomatic Complexity + Individual Path
</commit_message>
<xml_diff>
--- a/docs/Lab03/Lab03_WBT_TCs_Form.xlsx
+++ b/docs/Lab03/Lab03_WBT_TCs_Form.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27932"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{614B0747-F6C0-4957-A497-8805580BE4B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BEBF744A-CFA0-449B-8631-6BF89E15843B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="22149" windowHeight="13200" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Statement" sheetId="1" r:id="rId1"/>
@@ -29,12 +29,15 @@
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="183" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="182" uniqueCount="103">
   <si>
     <t>VVSS, Info Romana, 2025-2026</t>
   </si>
@@ -156,13 +159,7 @@
     <t>F02_P01</t>
   </si>
   <si>
-    <t>1 - 2(F) - …</t>
-  </si>
-  <si>
     <t>F02_P02</t>
-  </si>
-  <si>
-    <t>1 - 2(T) - …</t>
   </si>
   <si>
     <t>F02_P03</t>
@@ -503,12 +500,48 @@
   <si>
     <t>Șandru Ștefan Tiberius</t>
   </si>
+  <si>
+    <t>19 - 15 + 2 = 6</t>
+  </si>
+  <si>
+    <t>5 + 1 = 6</t>
+  </si>
+  <si>
+    <t>F02_P04</t>
+  </si>
+  <si>
+    <t>F02_P05</t>
+  </si>
+  <si>
+    <t>F02_P06</t>
+  </si>
+  <si>
+    <t>1 - 2(F) - 4 - 5(F) - 14 - 15</t>
+  </si>
+  <si>
+    <t>1 - 2(T) - 3 - 15</t>
+  </si>
+  <si>
+    <t>1 - 2(F) - 4 - 5(T) - 6 - 7(T) - 8 - 15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 - 2(F) - 4 - 5(T) - 6 - 7(F) - 9(T) - 10 - 15 </t>
+  </si>
+  <si>
+    <t>1 - 2(F) - 4 - 5(T) - 6 - 7(F) - 9(F) - 11(T) - 12 - 15</t>
+  </si>
+  <si>
+    <t>1 - 2(F) - 4 - 5(T) - 6 - 7(F) - 9(F) - 11(F) - 13 - 5(F) - 14 - 15</t>
+  </si>
+  <si>
+    <t>F02. Calcularea totalului unei comenzi</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -643,6 +676,12 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="13">
     <fill>
@@ -1181,7 +1220,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="109">
+  <cellXfs count="111">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1274,206 +1313,212 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="12" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="12" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="7" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="11" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="11" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="11" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="10" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="10" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="11" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="12" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="12" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1494,80 +1539,6 @@
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>621030</xdr:colOff>
-      <xdr:row>8</xdr:row>
-      <xdr:rowOff>125730</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>15</xdr:col>
-      <xdr:colOff>194310</xdr:colOff>
-      <xdr:row>31</xdr:row>
-      <xdr:rowOff>87630</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="6188" name="Picture 4">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0100-00002C180000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:srcRect/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr bwMode="auto">
-        <a:xfrm>
-          <a:off x="5208270" y="1588770"/>
-          <a:ext cx="4724400" cy="4168140"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:extLst>
-          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-              <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
-              </a:solidFill>
-            </a14:hiddenFill>
-          </a:ext>
-          <a:ext uri="{91240B29-F687-4F45-9708-019B960494DF}">
-            <a14:hiddenLine xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" w="9525">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:miter lim="800000"/>
-              <a:headEnd/>
-              <a:tailEnd/>
-            </a14:hiddenLine>
-          </a:ext>
-        </a:extLst>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>0</xdr:col>
@@ -1595,7 +1566,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -1604,6 +1575,50 @@
         <a:xfrm>
           <a:off x="571499" y="1321127"/>
           <a:ext cx="3999343" cy="2658843"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>1</xdr:colOff>
+      <xdr:row>35</xdr:row>
+      <xdr:rowOff>138565</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="Picture 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{58F62809-31FE-4830-36F3-732ED6CA8A1D}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="5083860" y="1667598"/>
+          <a:ext cx="4377447" cy="4956073"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1906,28 +1921,28 @@
     <tabColor theme="5" tint="0.59999389629810485"/>
   </sheetPr>
   <dimension ref="B1:P20"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.84375" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="13" max="13" width="14" customWidth="1"/>
-    <col min="14" max="14" width="11.140625" customWidth="1"/>
-    <col min="15" max="15" width="25.85546875" customWidth="1"/>
+    <col min="14" max="14" width="11.15234375" customWidth="1"/>
+    <col min="15" max="15" width="25.84375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="1" spans="2:16" x14ac:dyDescent="0.4">
       <c r="B1" s="12"/>
-      <c r="D1" s="66" t="s">
+      <c r="D1" s="43" t="s">
         <v>0</v>
       </c>
-      <c r="E1" s="67"/>
-      <c r="F1" s="67"/>
-      <c r="G1" s="68"/>
-    </row>
-    <row r="2" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="E1" s="44"/>
+      <c r="F1" s="44"/>
+      <c r="G1" s="45"/>
+    </row>
+    <row r="2" spans="2:16" x14ac:dyDescent="0.4">
       <c r="B2" s="41" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:16" x14ac:dyDescent="0.4">
       <c r="B4" s="1" t="s">
         <v>2</v>
       </c>
@@ -1937,7 +1952,7 @@
       <c r="O4" s="5"/>
       <c r="P4" s="5"/>
     </row>
-    <row r="5" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:16" x14ac:dyDescent="0.4">
       <c r="B5" s="1" t="s">
         <v>4</v>
       </c>
@@ -1947,7 +1962,7 @@
       <c r="O5" s="37"/>
       <c r="P5" s="37"/>
     </row>
-    <row r="6" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:16" x14ac:dyDescent="0.4">
       <c r="B6" s="1" t="s">
         <v>6</v>
       </c>
@@ -1959,7 +1974,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:16" x14ac:dyDescent="0.4">
       <c r="B7" s="1"/>
       <c r="C7" s="1"/>
       <c r="D7" s="1"/>
@@ -1968,13 +1983,13 @@
         <v>9</v>
       </c>
       <c r="O7" s="29" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="P7" s="29">
         <v>236</v>
       </c>
     </row>
-    <row r="8" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:16" x14ac:dyDescent="0.4">
       <c r="B8" s="1"/>
       <c r="C8" s="1"/>
       <c r="D8" s="1"/>
@@ -1983,15 +1998,15 @@
         <v>10</v>
       </c>
       <c r="O8" s="29" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="P8" s="29">
         <v>236</v>
       </c>
     </row>
-    <row r="9" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:16" x14ac:dyDescent="0.4">
       <c r="B9" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="C9" s="1"/>
       <c r="D9" s="1"/>
@@ -2000,37 +2015,37 @@
         <v>11</v>
       </c>
       <c r="O9" s="29" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="P9" s="29">
         <v>236</v>
       </c>
     </row>
-    <row r="10" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:16" x14ac:dyDescent="0.4">
       <c r="B10" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="C10" s="1"/>
       <c r="D10" s="1"/>
       <c r="E10" s="1"/>
     </row>
-    <row r="11" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:16" x14ac:dyDescent="0.4">
       <c r="B11" s="39" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="C11" s="1"/>
       <c r="D11" s="1"/>
       <c r="E11" s="1"/>
     </row>
-    <row r="12" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:16" x14ac:dyDescent="0.4">
       <c r="C12" s="1"/>
       <c r="D12" s="1"/>
       <c r="E12" s="1"/>
     </row>
-    <row r="19" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:2" x14ac:dyDescent="0.4">
       <c r="B19" s="1"/>
     </row>
-    <row r="20" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:2" x14ac:dyDescent="0.4">
       <c r="B20" s="1"/>
     </row>
   </sheetData>
@@ -2048,367 +2063,376 @@
     <tabColor theme="7" tint="0.59999389629810485"/>
   </sheetPr>
   <dimension ref="B1:T24"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.84375" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="2" max="2" width="10" customWidth="1"/>
-    <col min="17" max="17" width="10.5703125" customWidth="1"/>
+    <col min="17" max="17" width="10.53515625" customWidth="1"/>
+    <col min="20" max="20" width="29.84375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="1" spans="2:20" x14ac:dyDescent="0.4">
       <c r="B1" s="12"/>
-      <c r="D1" s="66" t="s">
+      <c r="D1" s="43" t="s">
         <v>0</v>
       </c>
-      <c r="E1" s="67"/>
-      <c r="F1" s="67"/>
-      <c r="G1" s="67"/>
-      <c r="H1" s="67"/>
-      <c r="I1" s="68"/>
-    </row>
-    <row r="3" spans="2:20" x14ac:dyDescent="0.25">
-      <c r="B3" s="87" t="s">
+      <c r="E1" s="44"/>
+      <c r="F1" s="44"/>
+      <c r="G1" s="44"/>
+      <c r="H1" s="44"/>
+      <c r="I1" s="45"/>
+    </row>
+    <row r="3" spans="2:20" x14ac:dyDescent="0.4">
+      <c r="B3" s="47" t="s">
         <v>12</v>
       </c>
-      <c r="C3" s="88"/>
-      <c r="D3" s="88"/>
-      <c r="E3" s="88"/>
-      <c r="F3" s="88"/>
-      <c r="G3" s="88"/>
-      <c r="H3" s="88"/>
-      <c r="I3" s="88"/>
-      <c r="J3" s="88"/>
-      <c r="K3" s="89"/>
-    </row>
-    <row r="6" spans="2:20" x14ac:dyDescent="0.25">
-      <c r="B6" s="66" t="s">
+      <c r="C3" s="48"/>
+      <c r="D3" s="48"/>
+      <c r="E3" s="48"/>
+      <c r="F3" s="48"/>
+      <c r="G3" s="48"/>
+      <c r="H3" s="48"/>
+      <c r="I3" s="48"/>
+      <c r="J3" s="48"/>
+      <c r="K3" s="49"/>
+    </row>
+    <row r="6" spans="2:20" x14ac:dyDescent="0.4">
+      <c r="B6" s="43" t="s">
         <v>13</v>
       </c>
-      <c r="C6" s="67"/>
-      <c r="D6" s="67"/>
-      <c r="E6" s="68"/>
+      <c r="C6" s="44"/>
+      <c r="D6" s="44"/>
+      <c r="E6" s="45"/>
       <c r="F6" s="33"/>
       <c r="G6" s="33"/>
-      <c r="I6" s="66" t="s">
+      <c r="I6" s="43" t="s">
         <v>14</v>
       </c>
-      <c r="J6" s="67"/>
-      <c r="K6" s="67"/>
-      <c r="L6" s="67"/>
-      <c r="M6" s="67"/>
-      <c r="N6" s="67"/>
-      <c r="O6" s="67"/>
-      <c r="Q6" s="66" t="s">
+      <c r="J6" s="44"/>
+      <c r="K6" s="44"/>
+      <c r="L6" s="44"/>
+      <c r="M6" s="44"/>
+      <c r="N6" s="44"/>
+      <c r="O6" s="44"/>
+      <c r="Q6" s="43" t="s">
         <v>15</v>
       </c>
-      <c r="R6" s="67"/>
-      <c r="S6" s="67"/>
-      <c r="T6" s="67"/>
-    </row>
-    <row r="8" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="R6" s="44"/>
+      <c r="S6" s="44"/>
+      <c r="T6" s="44"/>
+    </row>
+    <row r="8" spans="2:20" x14ac:dyDescent="0.4">
       <c r="B8" s="34" t="s">
         <v>16</v>
       </c>
-      <c r="C8" s="99" t="s">
+      <c r="C8" s="61" t="s">
         <v>17</v>
       </c>
-      <c r="D8" s="99"/>
-      <c r="E8" s="99"/>
+      <c r="D8" s="61"/>
+      <c r="E8" s="61"/>
       <c r="F8" s="35"/>
       <c r="G8" s="35"/>
       <c r="I8" s="12" t="s">
         <v>18</v>
       </c>
-      <c r="Q8" s="86" t="s">
+      <c r="Q8" s="60" t="s">
         <v>19</v>
       </c>
-      <c r="R8" s="86"/>
-      <c r="S8" s="86"/>
-      <c r="T8" s="36" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="9" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="R8" s="60"/>
+      <c r="S8" s="60"/>
+      <c r="T8" s="36">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9" spans="2:20" x14ac:dyDescent="0.4">
       <c r="B9" s="37" t="s">
         <v>21</v>
       </c>
-      <c r="C9" s="85" t="s">
-        <v>20</v>
-      </c>
-      <c r="D9" s="85"/>
-      <c r="E9" s="85"/>
+      <c r="C9" s="50" t="s">
+        <v>20</v>
+      </c>
+      <c r="D9" s="50"/>
+      <c r="E9" s="50"/>
       <c r="F9" s="38"/>
       <c r="G9" s="38"/>
       <c r="I9" s="40"/>
-      <c r="Q9" s="86" t="s">
+      <c r="Q9" s="60" t="s">
         <v>22</v>
       </c>
-      <c r="R9" s="86"/>
-      <c r="S9" s="86"/>
+      <c r="R9" s="60"/>
+      <c r="S9" s="60"/>
       <c r="T9" s="36" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="10" spans="2:20" x14ac:dyDescent="0.25">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="10" spans="2:20" x14ac:dyDescent="0.4">
       <c r="B10" s="37" t="s">
         <v>23</v>
       </c>
-      <c r="C10" s="85" t="s">
-        <v>20</v>
-      </c>
-      <c r="D10" s="85"/>
-      <c r="E10" s="85"/>
+      <c r="C10" s="50" t="s">
+        <v>20</v>
+      </c>
+      <c r="D10" s="50"/>
+      <c r="E10" s="50"/>
       <c r="F10" s="38"/>
       <c r="G10" s="38"/>
-      <c r="I10" s="90" t="s">
+      <c r="I10" s="51" t="s">
         <v>24</v>
       </c>
-      <c r="J10" s="91"/>
-      <c r="K10" s="91"/>
-      <c r="L10" s="91"/>
-      <c r="M10" s="91"/>
-      <c r="N10" s="91"/>
-      <c r="O10" s="92"/>
-      <c r="Q10" s="86" t="s">
+      <c r="J10" s="52"/>
+      <c r="K10" s="52"/>
+      <c r="L10" s="52"/>
+      <c r="M10" s="52"/>
+      <c r="N10" s="52"/>
+      <c r="O10" s="53"/>
+      <c r="Q10" s="60" t="s">
         <v>25</v>
       </c>
-      <c r="R10" s="86" t="s">
+      <c r="R10" s="60" t="s">
         <v>26</v>
       </c>
-      <c r="S10" s="86"/>
+      <c r="S10" s="60"/>
       <c r="T10" s="36" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="11" spans="2:20" x14ac:dyDescent="0.25">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="11" spans="2:20" x14ac:dyDescent="0.4">
       <c r="B11" s="37" t="s">
         <v>27</v>
       </c>
-      <c r="C11" s="85" t="s">
-        <v>20</v>
-      </c>
-      <c r="D11" s="85"/>
-      <c r="E11" s="85"/>
+      <c r="C11" s="50" t="s">
+        <v>20</v>
+      </c>
+      <c r="D11" s="50"/>
+      <c r="E11" s="50"/>
       <c r="F11" s="38"/>
       <c r="G11" s="38"/>
-      <c r="I11" s="93"/>
-      <c r="J11" s="94"/>
-      <c r="K11" s="94"/>
-      <c r="L11" s="94"/>
-      <c r="M11" s="94"/>
-      <c r="N11" s="94"/>
-      <c r="O11" s="95"/>
-    </row>
-    <row r="12" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="I11" s="54"/>
+      <c r="J11" s="55"/>
+      <c r="K11" s="55"/>
+      <c r="L11" s="55"/>
+      <c r="M11" s="55"/>
+      <c r="N11" s="55"/>
+      <c r="O11" s="56"/>
+    </row>
+    <row r="12" spans="2:20" x14ac:dyDescent="0.4">
       <c r="B12" s="37" t="s">
         <v>28</v>
       </c>
-      <c r="C12" s="85" t="s">
-        <v>20</v>
-      </c>
-      <c r="D12" s="85"/>
-      <c r="E12" s="85"/>
+      <c r="C12" s="50" t="s">
+        <v>20</v>
+      </c>
+      <c r="D12" s="50"/>
+      <c r="E12" s="50"/>
       <c r="F12" s="38"/>
       <c r="G12" s="38"/>
-      <c r="I12" s="93"/>
-      <c r="J12" s="94"/>
-      <c r="K12" s="94"/>
-      <c r="L12" s="94"/>
-      <c r="M12" s="94"/>
-      <c r="N12" s="94"/>
-      <c r="O12" s="95"/>
-    </row>
-    <row r="13" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="I12" s="54"/>
+      <c r="J12" s="55"/>
+      <c r="K12" s="55"/>
+      <c r="L12" s="55"/>
+      <c r="M12" s="55"/>
+      <c r="N12" s="55"/>
+      <c r="O12" s="56"/>
+    </row>
+    <row r="13" spans="2:20" x14ac:dyDescent="0.4">
       <c r="B13" s="37" t="s">
         <v>29</v>
       </c>
-      <c r="C13" s="85" t="s">
-        <v>20</v>
-      </c>
-      <c r="D13" s="85"/>
-      <c r="E13" s="85"/>
+      <c r="C13" s="50" t="s">
+        <v>20</v>
+      </c>
+      <c r="D13" s="50"/>
+      <c r="E13" s="50"/>
       <c r="F13" s="38"/>
       <c r="G13" s="38"/>
-      <c r="I13" s="93"/>
-      <c r="J13" s="94"/>
-      <c r="K13" s="94"/>
-      <c r="L13" s="94"/>
-      <c r="M13" s="94"/>
-      <c r="N13" s="94"/>
-      <c r="O13" s="95"/>
-      <c r="Q13" s="66" t="s">
+      <c r="I13" s="54"/>
+      <c r="J13" s="55"/>
+      <c r="K13" s="55"/>
+      <c r="L13" s="55"/>
+      <c r="M13" s="55"/>
+      <c r="N13" s="55"/>
+      <c r="O13" s="56"/>
+      <c r="Q13" s="43" t="s">
         <v>30</v>
       </c>
-      <c r="R13" s="67"/>
-      <c r="S13" s="67"/>
-      <c r="T13" s="67"/>
-    </row>
-    <row r="14" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="R13" s="44"/>
+      <c r="S13" s="44"/>
+      <c r="T13" s="44"/>
+    </row>
+    <row r="14" spans="2:20" x14ac:dyDescent="0.4">
       <c r="B14" s="37" t="s">
         <v>28</v>
       </c>
-      <c r="C14" s="85" t="s">
-        <v>20</v>
-      </c>
-      <c r="D14" s="85"/>
-      <c r="E14" s="85"/>
+      <c r="C14" s="50" t="s">
+        <v>20</v>
+      </c>
+      <c r="D14" s="50"/>
+      <c r="E14" s="50"/>
       <c r="F14" s="38"/>
       <c r="G14" s="38"/>
-      <c r="I14" s="93"/>
-      <c r="J14" s="94"/>
-      <c r="K14" s="94"/>
-      <c r="L14" s="94"/>
-      <c r="M14" s="94"/>
-      <c r="N14" s="94"/>
-      <c r="O14" s="95"/>
-    </row>
-    <row r="15" spans="2:20" x14ac:dyDescent="0.25">
-      <c r="I15" s="93"/>
-      <c r="J15" s="94"/>
-      <c r="K15" s="94"/>
-      <c r="L15" s="94"/>
-      <c r="M15" s="94"/>
-      <c r="N15" s="94"/>
-      <c r="O15" s="95"/>
+      <c r="I14" s="54"/>
+      <c r="J14" s="55"/>
+      <c r="K14" s="55"/>
+      <c r="L14" s="55"/>
+      <c r="M14" s="55"/>
+      <c r="N14" s="55"/>
+      <c r="O14" s="56"/>
+    </row>
+    <row r="15" spans="2:20" x14ac:dyDescent="0.4">
+      <c r="I15" s="54"/>
+      <c r="J15" s="55"/>
+      <c r="K15" s="55"/>
+      <c r="L15" s="55"/>
+      <c r="M15" s="55"/>
+      <c r="N15" s="55"/>
+      <c r="O15" s="56"/>
       <c r="Q15" s="34" t="s">
         <v>31</v>
       </c>
-      <c r="R15" s="99" t="s">
+      <c r="R15" s="61" t="s">
         <v>32</v>
       </c>
-      <c r="S15" s="99"/>
-      <c r="T15" s="99"/>
-    </row>
-    <row r="16" spans="2:20" x14ac:dyDescent="0.25">
-      <c r="I16" s="93"/>
-      <c r="J16" s="94"/>
-      <c r="K16" s="94"/>
-      <c r="L16" s="94"/>
-      <c r="M16" s="94"/>
-      <c r="N16" s="94"/>
-      <c r="O16" s="95"/>
+      <c r="S15" s="61"/>
+      <c r="T15" s="61"/>
+    </row>
+    <row r="16" spans="2:20" x14ac:dyDescent="0.4">
+      <c r="I16" s="54"/>
+      <c r="J16" s="55"/>
+      <c r="K16" s="55"/>
+      <c r="L16" s="55"/>
+      <c r="M16" s="55"/>
+      <c r="N16" s="55"/>
+      <c r="O16" s="56"/>
       <c r="Q16" s="37" t="s">
         <v>33</v>
       </c>
-      <c r="R16" s="84" t="s">
+      <c r="R16" s="46" t="s">
+        <v>96</v>
+      </c>
+      <c r="S16" s="46"/>
+      <c r="T16" s="46"/>
+    </row>
+    <row r="17" spans="9:20" x14ac:dyDescent="0.4">
+      <c r="I17" s="54"/>
+      <c r="J17" s="55"/>
+      <c r="K17" s="55"/>
+      <c r="L17" s="55"/>
+      <c r="M17" s="55"/>
+      <c r="N17" s="55"/>
+      <c r="O17" s="56"/>
+      <c r="Q17" s="37" t="s">
         <v>34</v>
       </c>
-      <c r="S16" s="84"/>
-      <c r="T16" s="84"/>
-    </row>
-    <row r="17" spans="9:20" x14ac:dyDescent="0.25">
-      <c r="I17" s="93"/>
-      <c r="J17" s="94"/>
-      <c r="K17" s="94"/>
-      <c r="L17" s="94"/>
-      <c r="M17" s="94"/>
-      <c r="N17" s="94"/>
-      <c r="O17" s="95"/>
-      <c r="Q17" s="37" t="s">
+      <c r="R17" s="46" t="s">
+        <v>97</v>
+      </c>
+      <c r="S17" s="46"/>
+      <c r="T17" s="46"/>
+    </row>
+    <row r="18" spans="9:20" x14ac:dyDescent="0.4">
+      <c r="I18" s="54"/>
+      <c r="J18" s="55"/>
+      <c r="K18" s="55"/>
+      <c r="L18" s="55"/>
+      <c r="M18" s="55"/>
+      <c r="N18" s="55"/>
+      <c r="O18" s="56"/>
+      <c r="Q18" s="37" t="s">
         <v>35</v>
       </c>
-      <c r="R17" s="84" t="s">
-        <v>36</v>
-      </c>
-      <c r="S17" s="84"/>
-      <c r="T17" s="84"/>
-    </row>
-    <row r="18" spans="9:20" x14ac:dyDescent="0.25">
-      <c r="I18" s="93"/>
-      <c r="J18" s="94"/>
-      <c r="K18" s="94"/>
-      <c r="L18" s="94"/>
-      <c r="M18" s="94"/>
-      <c r="N18" s="94"/>
-      <c r="O18" s="95"/>
-      <c r="Q18" s="37" t="s">
-        <v>37</v>
-      </c>
-      <c r="R18" s="84" t="s">
-        <v>20</v>
-      </c>
-      <c r="S18" s="84"/>
-      <c r="T18" s="84"/>
-    </row>
-    <row r="19" spans="9:20" x14ac:dyDescent="0.25">
-      <c r="I19" s="93"/>
-      <c r="J19" s="94"/>
-      <c r="K19" s="94"/>
-      <c r="L19" s="94"/>
-      <c r="M19" s="94"/>
-      <c r="N19" s="94"/>
-      <c r="O19" s="95"/>
+      <c r="R18" s="46" t="s">
+        <v>98</v>
+      </c>
+      <c r="S18" s="46"/>
+      <c r="T18" s="46"/>
+    </row>
+    <row r="19" spans="9:20" x14ac:dyDescent="0.4">
+      <c r="I19" s="54"/>
+      <c r="J19" s="55"/>
+      <c r="K19" s="55"/>
+      <c r="L19" s="55"/>
+      <c r="M19" s="55"/>
+      <c r="N19" s="55"/>
+      <c r="O19" s="56"/>
       <c r="Q19" s="37" t="s">
-        <v>28</v>
-      </c>
-      <c r="R19" s="84" t="s">
-        <v>20</v>
-      </c>
-      <c r="S19" s="84"/>
-      <c r="T19" s="84"/>
-    </row>
-    <row r="20" spans="9:20" x14ac:dyDescent="0.25">
-      <c r="I20" s="93"/>
-      <c r="J20" s="94"/>
-      <c r="K20" s="94"/>
-      <c r="L20" s="94"/>
-      <c r="M20" s="94"/>
-      <c r="N20" s="94"/>
-      <c r="O20" s="95"/>
-      <c r="Q20" s="37" t="s">
-        <v>29</v>
-      </c>
-      <c r="R20" s="84" t="s">
-        <v>20</v>
-      </c>
-      <c r="S20" s="84"/>
-      <c r="T20" s="84"/>
-    </row>
-    <row r="21" spans="9:20" x14ac:dyDescent="0.25">
-      <c r="I21" s="93"/>
-      <c r="J21" s="94"/>
-      <c r="K21" s="94"/>
-      <c r="L21" s="94"/>
-      <c r="M21" s="94"/>
-      <c r="N21" s="94"/>
-      <c r="O21" s="95"/>
-      <c r="Q21" s="37" t="s">
-        <v>28</v>
-      </c>
-      <c r="R21" s="84" t="s">
-        <v>20</v>
-      </c>
-      <c r="S21" s="84"/>
-      <c r="T21" s="84"/>
-    </row>
-    <row r="22" spans="9:20" x14ac:dyDescent="0.25">
-      <c r="I22" s="93"/>
-      <c r="J22" s="94"/>
-      <c r="K22" s="94"/>
-      <c r="L22" s="94"/>
-      <c r="M22" s="94"/>
-      <c r="N22" s="94"/>
-      <c r="O22" s="95"/>
-    </row>
-    <row r="23" spans="9:20" x14ac:dyDescent="0.25">
-      <c r="I23" s="93"/>
-      <c r="J23" s="94"/>
-      <c r="K23" s="94"/>
-      <c r="L23" s="94"/>
-      <c r="M23" s="94"/>
-      <c r="N23" s="94"/>
-      <c r="O23" s="95"/>
-    </row>
-    <row r="24" spans="9:20" x14ac:dyDescent="0.25">
-      <c r="I24" s="96"/>
-      <c r="J24" s="97"/>
-      <c r="K24" s="97"/>
-      <c r="L24" s="97"/>
-      <c r="M24" s="97"/>
-      <c r="N24" s="97"/>
-      <c r="O24" s="98"/>
+        <v>93</v>
+      </c>
+      <c r="R19" s="46" t="s">
+        <v>99</v>
+      </c>
+      <c r="S19" s="46"/>
+      <c r="T19" s="46"/>
+    </row>
+    <row r="20" spans="9:20" x14ac:dyDescent="0.4">
+      <c r="I20" s="54"/>
+      <c r="J20" s="55"/>
+      <c r="K20" s="55"/>
+      <c r="L20" s="55"/>
+      <c r="M20" s="55"/>
+      <c r="N20" s="55"/>
+      <c r="O20" s="56"/>
+      <c r="Q20" s="42" t="s">
+        <v>94</v>
+      </c>
+      <c r="R20" s="46" t="s">
+        <v>100</v>
+      </c>
+      <c r="S20" s="46"/>
+      <c r="T20" s="46"/>
+    </row>
+    <row r="21" spans="9:20" x14ac:dyDescent="0.4">
+      <c r="I21" s="54"/>
+      <c r="J21" s="55"/>
+      <c r="K21" s="55"/>
+      <c r="L21" s="55"/>
+      <c r="M21" s="55"/>
+      <c r="N21" s="55"/>
+      <c r="O21" s="56"/>
+      <c r="Q21" s="42" t="s">
+        <v>95</v>
+      </c>
+      <c r="R21" s="46" t="s">
+        <v>101</v>
+      </c>
+      <c r="S21" s="46"/>
+      <c r="T21" s="46"/>
+    </row>
+    <row r="22" spans="9:20" x14ac:dyDescent="0.4">
+      <c r="I22" s="54"/>
+      <c r="J22" s="55"/>
+      <c r="K22" s="55"/>
+      <c r="L22" s="55"/>
+      <c r="M22" s="55"/>
+      <c r="N22" s="55"/>
+      <c r="O22" s="56"/>
+    </row>
+    <row r="23" spans="9:20" x14ac:dyDescent="0.4">
+      <c r="I23" s="54"/>
+      <c r="J23" s="55"/>
+      <c r="K23" s="55"/>
+      <c r="L23" s="55"/>
+      <c r="M23" s="55"/>
+      <c r="N23" s="55"/>
+      <c r="O23" s="56"/>
+    </row>
+    <row r="24" spans="9:20" x14ac:dyDescent="0.4">
+      <c r="I24" s="57"/>
+      <c r="J24" s="58"/>
+      <c r="K24" s="58"/>
+      <c r="L24" s="58"/>
+      <c r="M24" s="58"/>
+      <c r="N24" s="58"/>
+      <c r="O24" s="59"/>
     </row>
   </sheetData>
   <mergeCells count="24">
+    <mergeCell ref="R18:T18"/>
+    <mergeCell ref="C9:E9"/>
+    <mergeCell ref="Q9:S9"/>
+    <mergeCell ref="R16:T16"/>
+    <mergeCell ref="C12:E12"/>
+    <mergeCell ref="C13:E13"/>
+    <mergeCell ref="Q13:T13"/>
+    <mergeCell ref="C14:E14"/>
     <mergeCell ref="D1:I1"/>
     <mergeCell ref="R20:T20"/>
     <mergeCell ref="R21:T21"/>
@@ -2425,15 +2449,8 @@
     <mergeCell ref="Q6:T6"/>
     <mergeCell ref="R17:T17"/>
     <mergeCell ref="R19:T19"/>
-    <mergeCell ref="R18:T18"/>
-    <mergeCell ref="C9:E9"/>
-    <mergeCell ref="Q9:S9"/>
-    <mergeCell ref="R16:T16"/>
-    <mergeCell ref="C12:E12"/>
-    <mergeCell ref="C13:E13"/>
-    <mergeCell ref="Q13:T13"/>
-    <mergeCell ref="C14:E14"/>
   </mergeCells>
+  <phoneticPr fontId="18" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <drawing r:id="rId2"/>
@@ -2446,254 +2463,254 @@
     <tabColor theme="7" tint="0.59999389629810485"/>
   </sheetPr>
   <dimension ref="B1:AB16"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.84375" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="2" max="2" width="12.28515625" customWidth="1"/>
-    <col min="3" max="4" width="18.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.140625" customWidth="1"/>
-    <col min="7" max="7" width="11.42578125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.140625" customWidth="1"/>
-    <col min="9" max="9" width="9.28515625" customWidth="1"/>
-    <col min="10" max="10" width="14.5703125" customWidth="1"/>
-    <col min="11" max="11" width="6.140625" customWidth="1"/>
-    <col min="12" max="12" width="6.42578125" customWidth="1"/>
+    <col min="2" max="2" width="12.3046875" customWidth="1"/>
+    <col min="3" max="4" width="18.15234375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="19.84375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.15234375" customWidth="1"/>
+    <col min="7" max="7" width="11.3828125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.15234375" customWidth="1"/>
+    <col min="9" max="9" width="9.3046875" customWidth="1"/>
+    <col min="10" max="10" width="14.53515625" customWidth="1"/>
+    <col min="11" max="11" width="6.15234375" customWidth="1"/>
+    <col min="12" max="12" width="6.3828125" customWidth="1"/>
     <col min="13" max="13" width="5" customWidth="1"/>
-    <col min="15" max="15" width="11.85546875" customWidth="1"/>
-    <col min="16" max="17" width="8.85546875" customWidth="1"/>
-    <col min="21" max="21" width="9.140625" customWidth="1"/>
-    <col min="22" max="24" width="2.140625" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="3.5703125" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="2.140625" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="4.140625" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="5.140625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="11.84375" customWidth="1"/>
+    <col min="16" max="17" width="8.84375" customWidth="1"/>
+    <col min="21" max="21" width="9.15234375" customWidth="1"/>
+    <col min="22" max="24" width="2.15234375" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="3.53515625" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="2.15234375" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="4.15234375" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="5.15234375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:28" x14ac:dyDescent="0.25">
+    <row r="1" spans="2:28" x14ac:dyDescent="0.4">
       <c r="B1" s="12"/>
-      <c r="D1" s="66" t="s">
+      <c r="D1" s="43" t="s">
         <v>0</v>
       </c>
-      <c r="E1" s="67"/>
-      <c r="F1" s="67"/>
-      <c r="G1" s="68"/>
-    </row>
-    <row r="3" spans="2:28" x14ac:dyDescent="0.25">
-      <c r="B3" s="87" t="s">
-        <v>12</v>
-      </c>
-      <c r="C3" s="88"/>
-      <c r="D3" s="88"/>
-      <c r="E3" s="88"/>
-      <c r="F3" s="89"/>
-    </row>
-    <row r="5" spans="2:28" x14ac:dyDescent="0.25">
+      <c r="E1" s="44"/>
+      <c r="F1" s="44"/>
+      <c r="G1" s="45"/>
+    </row>
+    <row r="3" spans="2:28" x14ac:dyDescent="0.4">
+      <c r="B3" s="110" t="s">
+        <v>102</v>
+      </c>
+      <c r="C3" s="48"/>
+      <c r="D3" s="48"/>
+      <c r="E3" s="48"/>
+      <c r="F3" s="49"/>
+    </row>
+    <row r="5" spans="2:28" x14ac:dyDescent="0.4">
       <c r="B5" s="11"/>
     </row>
-    <row r="6" spans="2:28" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B6" s="106" t="s">
+    <row r="6" spans="2:28" ht="15.9" x14ac:dyDescent="0.4">
+      <c r="B6" s="62" t="s">
+        <v>36</v>
+      </c>
+      <c r="C6" s="62" t="s">
+        <v>37</v>
+      </c>
+      <c r="D6" s="63" t="s">
         <v>38</v>
       </c>
-      <c r="C6" s="106" t="s">
+      <c r="E6" s="62" t="s">
         <v>39</v>
       </c>
-      <c r="D6" s="107" t="s">
+      <c r="F6" s="62"/>
+      <c r="G6" s="62"/>
+      <c r="H6" s="62"/>
+      <c r="I6" s="62"/>
+      <c r="J6" s="62"/>
+      <c r="K6" s="62"/>
+      <c r="L6" s="62"/>
+      <c r="M6" s="62"/>
+      <c r="N6" s="62"/>
+      <c r="O6" s="62"/>
+      <c r="P6" s="62"/>
+      <c r="Q6" s="62"/>
+      <c r="R6" s="62"/>
+      <c r="S6" s="62"/>
+      <c r="T6" s="62"/>
+      <c r="U6" s="62"/>
+      <c r="V6" s="62"/>
+      <c r="W6" s="62"/>
+      <c r="X6" s="62"/>
+      <c r="Y6" s="62"/>
+      <c r="Z6" s="62"/>
+      <c r="AA6" s="62"/>
+      <c r="AB6" s="62"/>
+    </row>
+    <row r="7" spans="2:28" ht="15.9" x14ac:dyDescent="0.4">
+      <c r="B7" s="62"/>
+      <c r="C7" s="62"/>
+      <c r="D7" s="64"/>
+      <c r="E7" s="70" t="s">
         <v>40</v>
       </c>
-      <c r="E6" s="106" t="s">
+      <c r="F7" s="69" t="s">
         <v>41</v>
       </c>
-      <c r="F6" s="106"/>
-      <c r="G6" s="106"/>
-      <c r="H6" s="106"/>
-      <c r="I6" s="106"/>
-      <c r="J6" s="106"/>
-      <c r="K6" s="106"/>
-      <c r="L6" s="106"/>
-      <c r="M6" s="106"/>
-      <c r="N6" s="106"/>
-      <c r="O6" s="106"/>
-      <c r="P6" s="106"/>
-      <c r="Q6" s="106"/>
-      <c r="R6" s="106"/>
-      <c r="S6" s="106"/>
-      <c r="T6" s="106"/>
-      <c r="U6" s="106"/>
-      <c r="V6" s="106"/>
-      <c r="W6" s="106"/>
-      <c r="X6" s="106"/>
-      <c r="Y6" s="106"/>
-      <c r="Z6" s="106"/>
-      <c r="AA6" s="106"/>
-      <c r="AB6" s="106"/>
-    </row>
-    <row r="7" spans="2:28" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B7" s="106"/>
-      <c r="C7" s="106"/>
-      <c r="D7" s="108"/>
-      <c r="E7" s="103" t="s">
+      <c r="G7" s="69"/>
+      <c r="H7" s="69"/>
+      <c r="I7" s="69"/>
+      <c r="J7" s="69"/>
+      <c r="K7" s="69"/>
+      <c r="L7" s="69"/>
+      <c r="M7" s="69"/>
+      <c r="N7" s="69"/>
+      <c r="O7" s="69"/>
+      <c r="P7" s="66" t="s">
         <v>42</v>
       </c>
-      <c r="F7" s="102" t="s">
+      <c r="Q7" s="66"/>
+      <c r="R7" s="66"/>
+      <c r="S7" s="66"/>
+      <c r="T7" s="66"/>
+      <c r="U7" s="66"/>
+      <c r="V7" s="65" t="s">
         <v>43</v>
       </c>
-      <c r="G7" s="102"/>
-      <c r="H7" s="102"/>
-      <c r="I7" s="102"/>
-      <c r="J7" s="102"/>
-      <c r="K7" s="102"/>
-      <c r="L7" s="102"/>
-      <c r="M7" s="102"/>
-      <c r="N7" s="102"/>
-      <c r="O7" s="102"/>
-      <c r="P7" s="104" t="s">
+      <c r="W7" s="65"/>
+      <c r="X7" s="65"/>
+      <c r="Y7" s="65"/>
+      <c r="Z7" s="65"/>
+      <c r="AA7" s="65"/>
+      <c r="AB7" s="65"/>
+    </row>
+    <row r="8" spans="2:28" ht="15.65" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="B8" s="62"/>
+      <c r="C8" s="67" t="s">
+        <v>20</v>
+      </c>
+      <c r="D8" s="67" t="s">
+        <v>20</v>
+      </c>
+      <c r="E8" s="70"/>
+      <c r="F8" s="69" t="s">
         <v>44</v>
       </c>
-      <c r="Q7" s="104"/>
-      <c r="R7" s="104"/>
-      <c r="S7" s="104"/>
-      <c r="T7" s="104"/>
-      <c r="U7" s="104"/>
-      <c r="V7" s="105" t="s">
+      <c r="G8" s="69"/>
+      <c r="H8" s="69" t="s">
         <v>45</v>
       </c>
-      <c r="W7" s="105"/>
-      <c r="X7" s="105"/>
-      <c r="Y7" s="105"/>
-      <c r="Z7" s="105"/>
-      <c r="AA7" s="105"/>
-      <c r="AB7" s="105"/>
-    </row>
-    <row r="8" spans="2:28" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B8" s="106"/>
-      <c r="C8" s="100" t="s">
-        <v>20</v>
-      </c>
-      <c r="D8" s="100" t="s">
-        <v>20</v>
-      </c>
-      <c r="E8" s="103"/>
-      <c r="F8" s="102" t="s">
+      <c r="I8" s="69"/>
+      <c r="J8" s="69" t="s">
         <v>46</v>
       </c>
-      <c r="G8" s="102"/>
-      <c r="H8" s="102" t="s">
+      <c r="K8" s="69"/>
+      <c r="L8" s="69" t="s">
+        <v>20</v>
+      </c>
+      <c r="M8" s="69"/>
+      <c r="N8" s="69" t="s">
         <v>47</v>
       </c>
-      <c r="I8" s="102"/>
-      <c r="J8" s="102" t="s">
+      <c r="O8" s="69"/>
+      <c r="P8" s="66" t="s">
+        <v>33</v>
+      </c>
+      <c r="Q8" s="66" t="s">
+        <v>34</v>
+      </c>
+      <c r="R8" s="66" t="s">
+        <v>20</v>
+      </c>
+      <c r="S8" s="66" t="s">
+        <v>20</v>
+      </c>
+      <c r="T8" s="66" t="s">
+        <v>20</v>
+      </c>
+      <c r="U8" s="66" t="s">
         <v>48</v>
       </c>
-      <c r="K8" s="102"/>
-      <c r="L8" s="102" t="s">
-        <v>20</v>
-      </c>
-      <c r="M8" s="102"/>
-      <c r="N8" s="102" t="s">
+      <c r="V8" s="65">
+        <v>0</v>
+      </c>
+      <c r="W8" s="65">
+        <v>1</v>
+      </c>
+      <c r="X8" s="65">
+        <v>2</v>
+      </c>
+      <c r="Y8" s="65" t="s">
         <v>49</v>
       </c>
-      <c r="O8" s="102"/>
-      <c r="P8" s="104" t="s">
-        <v>33</v>
-      </c>
-      <c r="Q8" s="104" t="s">
-        <v>35</v>
-      </c>
-      <c r="R8" s="104" t="s">
-        <v>20</v>
-      </c>
-      <c r="S8" s="104" t="s">
-        <v>20</v>
-      </c>
-      <c r="T8" s="104" t="s">
-        <v>20</v>
-      </c>
-      <c r="U8" s="104" t="s">
+      <c r="Z8" s="65" t="s">
         <v>50</v>
       </c>
-      <c r="V8" s="105">
-        <v>0</v>
-      </c>
-      <c r="W8" s="105">
-        <v>1</v>
-      </c>
-      <c r="X8" s="105">
-        <v>2</v>
-      </c>
-      <c r="Y8" s="105" t="s">
+      <c r="AA8" s="65" t="s">
         <v>51</v>
       </c>
-      <c r="Z8" s="105" t="s">
+      <c r="AB8" s="65" t="s">
         <v>52</v>
       </c>
-      <c r="AA8" s="105" t="s">
+    </row>
+    <row r="9" spans="2:28" ht="15.9" x14ac:dyDescent="0.4">
+      <c r="B9" s="62"/>
+      <c r="C9" s="68"/>
+      <c r="D9" s="68"/>
+      <c r="E9" s="70"/>
+      <c r="F9" s="13" t="s">
         <v>53</v>
       </c>
-      <c r="AB8" s="105" t="s">
+      <c r="G9" s="13" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="9" spans="2:28" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B9" s="106"/>
-      <c r="C9" s="101"/>
-      <c r="D9" s="101"/>
-      <c r="E9" s="103"/>
-      <c r="F9" s="13" t="s">
+      <c r="H9" s="13" t="s">
+        <v>53</v>
+      </c>
+      <c r="I9" s="13" t="s">
+        <v>54</v>
+      </c>
+      <c r="J9" s="13" t="s">
+        <v>53</v>
+      </c>
+      <c r="K9" s="13" t="s">
+        <v>54</v>
+      </c>
+      <c r="L9" s="13" t="s">
+        <v>53</v>
+      </c>
+      <c r="M9" s="13" t="s">
+        <v>54</v>
+      </c>
+      <c r="N9" s="13" t="s">
+        <v>53</v>
+      </c>
+      <c r="O9" s="13" t="s">
+        <v>54</v>
+      </c>
+      <c r="P9" s="66"/>
+      <c r="Q9" s="66"/>
+      <c r="R9" s="66"/>
+      <c r="S9" s="66"/>
+      <c r="T9" s="66"/>
+      <c r="U9" s="66"/>
+      <c r="V9" s="65"/>
+      <c r="W9" s="65"/>
+      <c r="X9" s="65"/>
+      <c r="Y9" s="65"/>
+      <c r="Z9" s="65"/>
+      <c r="AA9" s="65"/>
+      <c r="AB9" s="65"/>
+    </row>
+    <row r="10" spans="2:28" ht="15.9" x14ac:dyDescent="0.4">
+      <c r="B10" s="14" t="s">
         <v>55</v>
       </c>
-      <c r="G9" s="13" t="s">
+      <c r="C10" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="D10" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="E10" s="16" t="s">
         <v>56</v>
-      </c>
-      <c r="H9" s="13" t="s">
-        <v>55</v>
-      </c>
-      <c r="I9" s="13" t="s">
-        <v>56</v>
-      </c>
-      <c r="J9" s="13" t="s">
-        <v>55</v>
-      </c>
-      <c r="K9" s="13" t="s">
-        <v>56</v>
-      </c>
-      <c r="L9" s="13" t="s">
-        <v>55</v>
-      </c>
-      <c r="M9" s="13" t="s">
-        <v>56</v>
-      </c>
-      <c r="N9" s="13" t="s">
-        <v>55</v>
-      </c>
-      <c r="O9" s="13" t="s">
-        <v>56</v>
-      </c>
-      <c r="P9" s="104"/>
-      <c r="Q9" s="104"/>
-      <c r="R9" s="104"/>
-      <c r="S9" s="104"/>
-      <c r="T9" s="104"/>
-      <c r="U9" s="104"/>
-      <c r="V9" s="105"/>
-      <c r="W9" s="105"/>
-      <c r="X9" s="105"/>
-      <c r="Y9" s="105"/>
-      <c r="Z9" s="105"/>
-      <c r="AA9" s="105"/>
-      <c r="AB9" s="105"/>
-    </row>
-    <row r="10" spans="2:28" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B10" s="14" t="s">
-        <v>57</v>
-      </c>
-      <c r="C10" s="14" t="s">
-        <v>20</v>
-      </c>
-      <c r="D10" s="15" t="s">
-        <v>20</v>
-      </c>
-      <c r="E10" s="16" t="s">
-        <v>58</v>
       </c>
       <c r="F10" s="17"/>
       <c r="G10" s="17"/>
@@ -2719,9 +2736,9 @@
       <c r="AA10" s="19"/>
       <c r="AB10" s="19"/>
     </row>
-    <row r="11" spans="2:28" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:28" ht="15.9" x14ac:dyDescent="0.4">
       <c r="B11" s="14" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C11" s="14" t="s">
         <v>20</v>
@@ -2754,7 +2771,7 @@
       <c r="AA11" s="19"/>
       <c r="AB11" s="19"/>
     </row>
-    <row r="12" spans="2:28" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:28" ht="15.9" x14ac:dyDescent="0.4">
       <c r="B12" s="14" t="s">
         <v>20</v>
       </c>
@@ -2785,7 +2802,7 @@
       <c r="AA12" s="19"/>
       <c r="AB12" s="19"/>
     </row>
-    <row r="13" spans="2:28" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:28" ht="15.9" x14ac:dyDescent="0.4">
       <c r="B13" s="14" t="s">
         <v>20</v>
       </c>
@@ -2816,7 +2833,7 @@
       <c r="AA13" s="19"/>
       <c r="AB13" s="19"/>
     </row>
-    <row r="14" spans="2:28" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:28" ht="15.9" x14ac:dyDescent="0.4">
       <c r="B14" s="14" t="s">
         <v>20</v>
       </c>
@@ -2847,7 +2864,7 @@
       <c r="AA14" s="19"/>
       <c r="AB14" s="19"/>
     </row>
-    <row r="15" spans="2:28" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:28" ht="15.9" x14ac:dyDescent="0.4">
       <c r="B15" s="14" t="s">
         <v>20</v>
       </c>
@@ -2878,11 +2895,25 @@
       <c r="AA15" s="19"/>
       <c r="AB15" s="19"/>
     </row>
-    <row r="16" spans="2:28" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:28" ht="15.9" x14ac:dyDescent="0.4">
       <c r="B16" s="22"/>
     </row>
   </sheetData>
   <mergeCells count="30">
+    <mergeCell ref="C8:C9"/>
+    <mergeCell ref="N8:O8"/>
+    <mergeCell ref="E7:E9"/>
+    <mergeCell ref="F7:O7"/>
+    <mergeCell ref="P7:U7"/>
+    <mergeCell ref="AB8:AB9"/>
+    <mergeCell ref="H8:I8"/>
+    <mergeCell ref="J8:K8"/>
+    <mergeCell ref="L8:M8"/>
+    <mergeCell ref="V8:V9"/>
+    <mergeCell ref="P8:P9"/>
+    <mergeCell ref="Q8:Q9"/>
+    <mergeCell ref="R8:R9"/>
+    <mergeCell ref="S8:S9"/>
     <mergeCell ref="D1:G1"/>
     <mergeCell ref="B3:F3"/>
     <mergeCell ref="B6:B9"/>
@@ -2899,20 +2930,6 @@
     <mergeCell ref="Y8:Y9"/>
     <mergeCell ref="T8:T9"/>
     <mergeCell ref="V7:AB7"/>
-    <mergeCell ref="AB8:AB9"/>
-    <mergeCell ref="H8:I8"/>
-    <mergeCell ref="J8:K8"/>
-    <mergeCell ref="L8:M8"/>
-    <mergeCell ref="V8:V9"/>
-    <mergeCell ref="P8:P9"/>
-    <mergeCell ref="Q8:Q9"/>
-    <mergeCell ref="R8:R9"/>
-    <mergeCell ref="S8:S9"/>
-    <mergeCell ref="C8:C9"/>
-    <mergeCell ref="N8:O8"/>
-    <mergeCell ref="E7:E9"/>
-    <mergeCell ref="F7:O7"/>
-    <mergeCell ref="P7:U7"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -2925,104 +2942,104 @@
     <tabColor theme="3" tint="0.59999389629810485"/>
   </sheetPr>
   <dimension ref="B1:N16"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.84375" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="3" max="3" width="7.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.15234375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.3046875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="9" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="16.140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.15234375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.84375" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="10" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="7.140625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="10.140625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="10.140625" customWidth="1"/>
-    <col min="13" max="13" width="16.140625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.28515625" customWidth="1"/>
+    <col min="10" max="10" width="7.15234375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="10.15234375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10.15234375" customWidth="1"/>
+    <col min="13" max="13" width="16.15234375" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="12.3046875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="1" spans="2:14" x14ac:dyDescent="0.4">
       <c r="B1" s="12"/>
-      <c r="D1" s="66" t="s">
+      <c r="D1" s="43" t="s">
         <v>0</v>
       </c>
-      <c r="E1" s="67"/>
-      <c r="F1" s="67"/>
-      <c r="G1" s="68"/>
-    </row>
-    <row r="3" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B3" s="69" t="s">
+      <c r="E1" s="44"/>
+      <c r="F1" s="44"/>
+      <c r="G1" s="45"/>
+    </row>
+    <row r="3" spans="2:14" x14ac:dyDescent="0.4">
+      <c r="B3" s="73" t="s">
+        <v>58</v>
+      </c>
+      <c r="C3" s="73"/>
+      <c r="D3" s="73"/>
+      <c r="E3" s="73"/>
+      <c r="F3" s="73"/>
+      <c r="G3" s="73"/>
+      <c r="H3" s="73"/>
+      <c r="I3" s="73"/>
+      <c r="J3" s="73"/>
+      <c r="K3" s="73"/>
+      <c r="L3" s="73"/>
+    </row>
+    <row r="4" spans="2:14" x14ac:dyDescent="0.4">
+      <c r="B4" s="74" t="s">
+        <v>59</v>
+      </c>
+      <c r="C4" s="83" t="s">
         <v>60</v>
       </c>
-      <c r="C3" s="69"/>
-      <c r="D3" s="69"/>
-      <c r="E3" s="69"/>
-      <c r="F3" s="69"/>
-      <c r="G3" s="69"/>
-      <c r="H3" s="69"/>
-      <c r="I3" s="69"/>
-      <c r="J3" s="69"/>
-      <c r="K3" s="69"/>
-      <c r="L3" s="69"/>
-    </row>
-    <row r="4" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B4" s="70" t="s">
+      <c r="D4" s="85" t="s">
         <v>61</v>
       </c>
-      <c r="C4" s="53" t="s">
+      <c r="E4" s="76" t="s">
         <v>62</v>
       </c>
-      <c r="D4" s="80" t="s">
+      <c r="F4" s="82"/>
+      <c r="G4" s="82"/>
+      <c r="H4" s="82"/>
+      <c r="I4" s="82"/>
+      <c r="J4" s="77"/>
+      <c r="K4" s="76" t="s">
         <v>63</v>
       </c>
-      <c r="E4" s="72" t="s">
+      <c r="L4" s="77"/>
+    </row>
+    <row r="5" spans="2:14" ht="15" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="B5" s="75"/>
+      <c r="C5" s="84"/>
+      <c r="D5" s="86"/>
+      <c r="E5" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="I5" s="78" t="s">
+        <v>20</v>
+      </c>
+      <c r="J5" s="79"/>
+      <c r="K5" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="F4" s="78"/>
-      <c r="G4" s="78"/>
-      <c r="H4" s="78"/>
-      <c r="I4" s="78"/>
-      <c r="J4" s="73"/>
-      <c r="K4" s="72" t="s">
+      <c r="L5" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="L4" s="73"/>
-    </row>
-    <row r="5" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="71"/>
-      <c r="C5" s="79"/>
-      <c r="D5" s="81"/>
-      <c r="E5" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="F5" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="G5" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="H5" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="I5" s="74" t="s">
-        <v>20</v>
-      </c>
-      <c r="J5" s="75"/>
-      <c r="K5" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="L5" s="2" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="6" spans="2:14" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="6" spans="2:14" ht="15" thickTop="1" x14ac:dyDescent="0.4">
       <c r="B6" s="23">
         <v>9</v>
       </c>
-      <c r="C6" s="76" t="s">
-        <v>68</v>
+      <c r="C6" s="80" t="s">
+        <v>66</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="E6" s="24" t="s">
         <v>20</v>
@@ -3036,10 +3053,10 @@
       <c r="H6" s="24" t="s">
         <v>20</v>
       </c>
-      <c r="I6" s="82" t="s">
-        <v>20</v>
-      </c>
-      <c r="J6" s="83"/>
+      <c r="I6" s="87" t="s">
+        <v>20</v>
+      </c>
+      <c r="J6" s="88"/>
       <c r="K6" s="24" t="s">
         <v>20</v>
       </c>
@@ -3047,13 +3064,13 @@
         <v>20</v>
       </c>
     </row>
-    <row r="7" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:14" x14ac:dyDescent="0.4">
       <c r="B7" s="23">
         <v>10</v>
       </c>
-      <c r="C7" s="76"/>
+      <c r="C7" s="80"/>
       <c r="D7" s="4" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="E7" s="23">
         <v>5</v>
@@ -3067,10 +3084,10 @@
       <c r="H7" s="23" t="s">
         <v>20</v>
       </c>
-      <c r="I7" s="72" t="s">
-        <v>20</v>
-      </c>
-      <c r="J7" s="73"/>
+      <c r="I7" s="76" t="s">
+        <v>20</v>
+      </c>
+      <c r="J7" s="77"/>
       <c r="K7" s="23" t="s">
         <v>20</v>
       </c>
@@ -3078,11 +3095,11 @@
         <v>20</v>
       </c>
     </row>
-    <row r="8" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:14" x14ac:dyDescent="0.4">
       <c r="B8" s="23">
         <v>11</v>
       </c>
-      <c r="C8" s="76"/>
+      <c r="C8" s="80"/>
       <c r="D8" s="10" t="s">
         <v>20</v>
       </c>
@@ -3098,10 +3115,10 @@
       <c r="H8" s="23" t="s">
         <v>20</v>
       </c>
-      <c r="I8" s="72" t="s">
-        <v>20</v>
-      </c>
-      <c r="J8" s="73"/>
+      <c r="I8" s="76" t="s">
+        <v>20</v>
+      </c>
+      <c r="J8" s="77"/>
       <c r="K8" s="23" t="s">
         <v>20</v>
       </c>
@@ -3109,11 +3126,11 @@
         <v>20</v>
       </c>
     </row>
-    <row r="9" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:14" x14ac:dyDescent="0.4">
       <c r="B9" s="23">
         <v>12</v>
       </c>
-      <c r="C9" s="76"/>
+      <c r="C9" s="80"/>
       <c r="D9" s="10" t="s">
         <v>20</v>
       </c>
@@ -3129,10 +3146,10 @@
       <c r="H9" s="23" t="s">
         <v>20</v>
       </c>
-      <c r="I9" s="72" t="s">
-        <v>20</v>
-      </c>
-      <c r="J9" s="73"/>
+      <c r="I9" s="76" t="s">
+        <v>20</v>
+      </c>
+      <c r="J9" s="77"/>
       <c r="K9" s="23" t="s">
         <v>20</v>
       </c>
@@ -3140,11 +3157,11 @@
         <v>20</v>
       </c>
     </row>
-    <row r="10" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:14" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="B10" s="2">
         <v>13</v>
       </c>
-      <c r="C10" s="77"/>
+      <c r="C10" s="81"/>
       <c r="D10" s="9" t="s">
         <v>20</v>
       </c>
@@ -3160,10 +3177,10 @@
       <c r="H10" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="I10" s="74" t="s">
-        <v>20</v>
-      </c>
-      <c r="J10" s="75"/>
+      <c r="I10" s="78" t="s">
+        <v>20</v>
+      </c>
+      <c r="J10" s="79"/>
       <c r="K10" s="2" t="s">
         <v>20</v>
       </c>
@@ -3171,7 +3188,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="11" spans="2:14" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:14" ht="15" thickTop="1" x14ac:dyDescent="0.4">
       <c r="B11" s="3"/>
       <c r="C11" s="3"/>
       <c r="D11" s="3"/>
@@ -3184,92 +3201,92 @@
       <c r="K11" s="3"/>
       <c r="L11" s="3"/>
     </row>
-    <row r="12" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:14" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="B12" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="K12" s="25"/>
+    </row>
+    <row r="13" spans="2:14" ht="15.45" thickTop="1" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="B13" s="71" t="s">
+        <v>69</v>
+      </c>
+      <c r="C13" s="72"/>
+      <c r="D13" s="72"/>
+      <c r="E13" s="72"/>
+      <c r="F13" s="89" t="s">
         <v>70</v>
       </c>
-      <c r="K12" s="25"/>
-    </row>
-    <row r="13" spans="2:14" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="58" t="s">
+      <c r="G13" s="90"/>
+      <c r="H13" s="71" t="s">
         <v>71</v>
       </c>
-      <c r="C13" s="59"/>
-      <c r="D13" s="59"/>
-      <c r="E13" s="59"/>
-      <c r="F13" s="50" t="s">
+      <c r="I13" s="72"/>
+      <c r="J13" s="72"/>
+      <c r="K13" s="72"/>
+      <c r="L13" s="99"/>
+      <c r="M13" s="104" t="s">
         <v>72</v>
       </c>
-      <c r="G13" s="51"/>
-      <c r="H13" s="58" t="s">
+      <c r="N13" s="105"/>
+    </row>
+    <row r="14" spans="2:14" ht="15" thickTop="1" x14ac:dyDescent="0.4">
+      <c r="B14" s="103" t="s">
         <v>73</v>
       </c>
-      <c r="I13" s="59"/>
-      <c r="J13" s="59"/>
-      <c r="K13" s="59"/>
-      <c r="L13" s="60"/>
-      <c r="M13" s="64" t="s">
+      <c r="C14" s="95" t="s">
         <v>74</v>
       </c>
-      <c r="N13" s="65"/>
-    </row>
-    <row r="14" spans="2:14" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="B14" s="42" t="s">
+      <c r="D14" s="95" t="s">
         <v>75</v>
       </c>
-      <c r="C14" s="44" t="s">
+      <c r="E14" s="107" t="s">
         <v>76</v>
       </c>
-      <c r="D14" s="44" t="s">
+      <c r="F14" s="92" t="s">
         <v>77</v>
       </c>
-      <c r="E14" s="46" t="s">
+      <c r="G14" s="91" t="s">
         <v>78</v>
       </c>
-      <c r="F14" s="48" t="s">
+      <c r="H14" s="93" t="s">
         <v>79</v>
       </c>
-      <c r="G14" s="52" t="s">
+      <c r="I14" s="95" t="s">
+        <v>73</v>
+      </c>
+      <c r="J14" s="95" t="s">
+        <v>74</v>
+      </c>
+      <c r="K14" s="97" t="s">
         <v>80</v>
       </c>
-      <c r="H14" s="54" t="s">
+      <c r="L14" s="100" t="s">
         <v>81</v>
       </c>
-      <c r="I14" s="44" t="s">
-        <v>75</v>
-      </c>
-      <c r="J14" s="44" t="s">
-        <v>76</v>
-      </c>
-      <c r="K14" s="56" t="s">
+      <c r="M14" s="102" t="s">
         <v>82</v>
       </c>
-      <c r="L14" s="61" t="s">
+      <c r="N14" s="83" t="s">
         <v>83</v>
       </c>
-      <c r="M14" s="63" t="s">
-        <v>84</v>
-      </c>
-      <c r="N14" s="53" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="15" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B15" s="43"/>
-      <c r="C15" s="45"/>
-      <c r="D15" s="45"/>
-      <c r="E15" s="47"/>
-      <c r="F15" s="49"/>
-      <c r="G15" s="52"/>
-      <c r="H15" s="55"/>
-      <c r="I15" s="45"/>
-      <c r="J15" s="45"/>
-      <c r="K15" s="57"/>
-      <c r="L15" s="62"/>
-      <c r="M15" s="42"/>
-      <c r="N15" s="48"/>
-    </row>
-    <row r="16" spans="2:14" x14ac:dyDescent="0.25">
+    </row>
+    <row r="15" spans="2:14" x14ac:dyDescent="0.4">
+      <c r="B15" s="106"/>
+      <c r="C15" s="96"/>
+      <c r="D15" s="96"/>
+      <c r="E15" s="108"/>
+      <c r="F15" s="109"/>
+      <c r="G15" s="91"/>
+      <c r="H15" s="94"/>
+      <c r="I15" s="96"/>
+      <c r="J15" s="96"/>
+      <c r="K15" s="98"/>
+      <c r="L15" s="101"/>
+      <c r="M15" s="103"/>
+      <c r="N15" s="92"/>
+    </row>
+    <row r="16" spans="2:14" x14ac:dyDescent="0.4">
       <c r="B16" s="29">
         <f>SUM(C16:D16)</f>
         <v>0</v>
@@ -3283,10 +3300,10 @@
       <c r="E16" s="27"/>
       <c r="F16" s="28"/>
       <c r="G16" s="8" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="H16" s="7" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="I16" s="29">
         <f>SUM(J16:K16)</f>
@@ -3300,7 +3317,7 @@
       </c>
       <c r="L16" s="31"/>
       <c r="M16" s="6" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="N16" s="32">
         <f>C16</f>
@@ -3309,6 +3326,21 @@
     </row>
   </sheetData>
   <mergeCells count="31">
+    <mergeCell ref="H13:L13"/>
+    <mergeCell ref="L14:L15"/>
+    <mergeCell ref="M14:M15"/>
+    <mergeCell ref="M13:N13"/>
+    <mergeCell ref="B14:B15"/>
+    <mergeCell ref="C14:C15"/>
+    <mergeCell ref="D14:D15"/>
+    <mergeCell ref="E14:E15"/>
+    <mergeCell ref="F14:F15"/>
+    <mergeCell ref="G14:G15"/>
+    <mergeCell ref="N14:N15"/>
+    <mergeCell ref="H14:H15"/>
+    <mergeCell ref="I14:I15"/>
+    <mergeCell ref="K14:K15"/>
+    <mergeCell ref="J14:J15"/>
     <mergeCell ref="B13:E13"/>
     <mergeCell ref="D1:G1"/>
     <mergeCell ref="B3:L3"/>
@@ -3325,21 +3357,6 @@
     <mergeCell ref="I10:J10"/>
     <mergeCell ref="I8:J8"/>
     <mergeCell ref="F13:G13"/>
-    <mergeCell ref="G14:G15"/>
-    <mergeCell ref="N14:N15"/>
-    <mergeCell ref="H14:H15"/>
-    <mergeCell ref="I14:I15"/>
-    <mergeCell ref="K14:K15"/>
-    <mergeCell ref="J14:J15"/>
-    <mergeCell ref="H13:L13"/>
-    <mergeCell ref="L14:L15"/>
-    <mergeCell ref="M14:M15"/>
-    <mergeCell ref="M13:N13"/>
-    <mergeCell ref="B14:B15"/>
-    <mergeCell ref="C14:C15"/>
-    <mergeCell ref="D14:D15"/>
-    <mergeCell ref="E14:E15"/>
-    <mergeCell ref="F14:F15"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -3347,6 +3364,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="301f98df-4edd-4096-94f8-2f8af3eee570">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="cbfc0213-1ef7-4e52-9599-c30bc1b3f3d7" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100E819BB071F23F542A5DF0E9C9037AD04" ma:contentTypeVersion="10" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="08d9df77a39a0ee87f79f9436c57bbce">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="301f98df-4edd-4096-94f8-2f8af3eee570" xmlns:ns3="cbfc0213-1ef7-4e52-9599-c30bc1b3f3d7" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="03dd79bc1474883a2d909db85c328b07" ns2:_="" ns3:_="">
     <xsd:import namespace="301f98df-4edd-4096-94f8-2f8af3eee570"/>
@@ -3535,27 +3572,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FA2F5940-EC19-4D08-A8C2-FA31EF734077}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="301f98df-4edd-4096-94f8-2f8af3eee570"/>
+    <ds:schemaRef ds:uri="cbfc0213-1ef7-4e52-9599-c30bc1b3f3d7"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="301f98df-4edd-4096-94f8-2f8af3eee570">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="cbfc0213-1ef7-4e52-9599-c30bc1b3f3d7" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EECFCB93-350B-4228-B7F4-DB12383611F2}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6B359A3C-84EA-4FDD-BB5C-023A91F35CC6}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3572,23 +3608,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EECFCB93-350B-4228-B7F4-DB12383611F2}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FA2F5940-EC19-4D08-A8C2-FA31EF734077}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="301f98df-4edd-4096-94f8-2f8af3eee570"/>
-    <ds:schemaRef ds:uri="cbfc0213-1ef7-4e52-9599-c30bc1b3f3d7"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>